<commit_message>
Savegarde des données page par page
</commit_message>
<xml_diff>
--- a/TimeTracker.xlsx
+++ b/TimeTracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Works\KungFu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E25269-61DB-4287-B5A9-614B4C30A41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4789D70D-720C-489E-86F1-CE22E5F11C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8988" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -207,8 +207,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C07780F6-4EDD-4593-9309-66544A000426}" name="Tableau1" displayName="Tableau1" ref="A1:E13" totalsRowCount="1" headerRowDxfId="11">
-  <autoFilter ref="A1:E12" xr:uid="{C07780F6-4EDD-4593-9309-66544A000426}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C07780F6-4EDD-4593-9309-66544A000426}" name="Tableau1" displayName="Tableau1" ref="A1:E14" totalsRowCount="1" headerRowDxfId="11">
+  <autoFilter ref="A1:E13" xr:uid="{C07780F6-4EDD-4593-9309-66544A000426}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{9CE1E16E-0A99-4229-9545-CEB505BEA2F7}" name="Jours" totalsRowLabel="Total" dataDxfId="10" totalsRowDxfId="3"/>
     <tableColumn id="2" xr3:uid="{3224133E-C10D-49BC-81D3-C06B33B14FB6}" name="Temps" totalsRowFunction="sum" dataDxfId="9" totalsRowDxfId="2"/>
@@ -504,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" style="3" customWidth="1"/>
@@ -763,18 +763,34 @@
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="3">
+        <v>46097</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2">
+        <v>30</v>
+      </c>
+      <c r="D13" s="2">
+        <f>Tableau1[[#This Row],[Temps]]*Tableau1[[#This Row],[Taux (horaire)]]</f>
+        <v>60</v>
+      </c>
+      <c r="J13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B14" s="1">
         <f>SUBTOTAL(109,Tableau1[Temps])</f>
-        <v>24</v>
-      </c>
-      <c r="D13" s="2">
+        <v>26</v>
+      </c>
+      <c r="D14" s="2">
         <f>SUBTOTAL(109,Tableau1[Prix])</f>
-        <v>750</v>
-      </c>
-      <c r="E13">
+        <v>810</v>
+      </c>
+      <c r="E14">
         <f>SUBTOTAL(103,Tableau1[Détails])</f>
         <v>9</v>
       </c>

</xml_diff>